<commit_message>
27/02/18 ultima ejecucion: 2026-02-18 actualizacion de credenciales
</commit_message>
<xml_diff>
--- a/cedulas.xlsx
+++ b/cedulas.xlsx
@@ -1,47 +1,62 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24701"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ContratosSuperflex\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2445A294-367D-4B5A-A78B-9FDFB3742939}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-11805" yWindow="8940" windowWidth="12150" windowHeight="11385" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
+    <sheet name="Hoja1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="3">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color rgb="FF000000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor rgb="FFFF0000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FF0000"/>
+        <bgColor rgb="00FF0000"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -57,64 +72,85 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+  <cellXfs count="4">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
+    <cellStyle name="Normal 2" xfId="1"/>
   </cellStyles>
-  <dxfs count="4">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -380,58 +416,36 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:A44"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A2:B4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="24.36328125" customWidth="1"/>
-    <col min="2" max="2" width="21.08984375" customWidth="1"/>
-    <col min="3" max="3" width="17.81640625" customWidth="1"/>
+    <col width="24.42578125" customWidth="1" min="1" max="1"/>
+    <col width="21.140625" customWidth="1" min="2" max="2"/>
+    <col width="17.85546875" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="2" ht="15.5" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="3" ht="15.5" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="13" ht="15.5" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="14" ht="15.5" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="15" ht="15.5" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="16" ht="15.5" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="17" ht="15.5" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="18" ht="15.5" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="19" ht="15.5" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="20" ht="15.5" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="21" ht="15.5" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="22" ht="15.5" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="23" ht="15.5" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="24" ht="15.5" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="25" ht="15.5" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="26" ht="15.5" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="27" ht="15.5" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="28" ht="15.5" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="29" ht="15.5" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="30" ht="15.5" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="31" ht="15.5" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="32" ht="15.5" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="33" ht="15.5" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="34" ht="15.5" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="35" ht="15.5" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="36" ht="15.5" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="37" ht="15.5" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="38" ht="15.5" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="39" ht="15.5" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="40" ht="15.5" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="41" ht="15.5" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="42" ht="15.5" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="43" ht="15.5" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="44" ht="15.5" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="2" ht="15.6" customHeight="1">
+      <c r="A2" s="3" t="n">
+        <v>68297670</v>
+      </c>
+    </row>
+    <row r="3" ht="15.6" customHeight="1">
+      <c r="A3" s="3" t="n">
+        <v>80155489</v>
+      </c>
+      <c r="B3" s="1" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="n">
+        <v>800159687</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="A7">
-    <cfRule type="cellIs" dxfId="3" priority="3" operator="equal">
-      <formula>31006459</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="4" operator="equal">
-      <formula>31006459</formula>
-    </cfRule>
-  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
 </worksheet>

</xml_diff>

<commit_message>
nueva funcionalidad envio de correo 15/05/2026 3:41pm
</commit_message>
<xml_diff>
--- a/cedulas.xlsx
+++ b/cedulas.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-11805" yWindow="8940" windowWidth="12150" windowHeight="11385" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" state="visible" r:id="rId1"/>
@@ -16,7 +16,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,16 +30,8 @@
       <color rgb="FF000000"/>
       <sz val="11"/>
     </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <u val="single"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -54,8 +46,20 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FF00FF00"/>
+        <bgColor rgb="FF00FF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00FF0000"/>
         <bgColor rgb="00FF0000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0000FF00"/>
+        <bgColor rgb="0000FF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -72,11 +76,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -421,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:B4"/>
+  <dimension ref="A2:A14"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="24.42578125" customWidth="1" min="1" max="1"/>
@@ -429,20 +434,69 @@
     <col width="17.85546875" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="2" ht="15.6" customHeight="1">
+    <row r="2">
       <c r="A2" s="3" t="n">
-        <v>68297670</v>
-      </c>
-    </row>
-    <row r="3" ht="15.6" customHeight="1">
-      <c r="A3" s="3" t="n">
         <v>80155489</v>
       </c>
-      <c r="B3" s="1" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="n">
+        <v>1001049512</v>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="n">
+      <c r="A4" s="4" t="n">
+        <v>1122512207</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="n">
+        <v>80109062</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="n">
+        <v>1121417451</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="n">
+        <v>1123140582</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="n">
+        <v>1234788097</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="n">
+        <v>1121851069</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="n">
+        <v>1122650938</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="n">
+        <v>40219614</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="n">
+        <v>1121840824</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="n">
         <v>800159687</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="n">
+        <v>1006720679</v>
       </c>
     </row>
   </sheetData>

</xml_diff>